<commit_message>
created seating leayout and several seat colours
</commit_message>
<xml_diff>
--- a/Time Plan.xlsx
+++ b/Time Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25svynarcht230_collyers_ac_uk/Documents/programming/Transfer Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19156623-1945-4D15-89AF-1B65381017BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{19156623-1945-4D15-89AF-1B65381017BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCF65993-33AA-4ABD-8164-32ED6B26E1A6}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -172,7 +172,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -206,6 +206,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -287,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -330,6 +354,14 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -773,7 +805,7 @@
       <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="14"/>
+      <c r="B4" s="26"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
@@ -787,8 +819,8 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="27"/>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
@@ -801,8 +833,8 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="22"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
@@ -829,8 +861,8 @@
       <c r="A8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="23"/>
       <c r="D8" s="16"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -844,8 +876,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="24"/>
       <c r="E9" s="15"/>
       <c r="F9" s="15"/>
       <c r="G9" s="15"/>
@@ -858,8 +890,8 @@
         <v>8</v>
       </c>
       <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="15"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
@@ -871,8 +903,8 @@
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="23"/>
       <c r="D11" s="15"/>
       <c r="E11" s="17"/>
       <c r="F11" s="15"/>
@@ -885,9 +917,9 @@
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
       <c r="E12" s="17"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
@@ -900,8 +932,8 @@
         <v>11</v>
       </c>
       <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="23"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
@@ -943,12 +975,12 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="24"/>
       <c r="J16" s="15"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -957,13 +989,13 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="D17" s="24"/>
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="24"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
@@ -975,9 +1007,9 @@
       <c r="E18" s="18"/>
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="24"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
@@ -1004,7 +1036,7 @@
       <c r="F20" s="14"/>
       <c r="G20" s="19"/>
       <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="I20" s="28"/>
       <c r="J20" s="14"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -1018,7 +1050,7 @@
       <c r="F21" s="15"/>
       <c r="G21" s="15"/>
       <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
+      <c r="I21" s="29"/>
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -1032,8 +1064,8 @@
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -1047,7 +1079,7 @@
       <c r="G23" s="15"/>
       <c r="H23" s="15"/>
       <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
+      <c r="J23" s="29"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -1061,7 +1093,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
+      <c r="J24" s="29"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -1075,7 +1107,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
+      <c r="J25" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1099,6 +1131,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
+      <UserInfo>
+        <DisplayName>Helen Browne</DisplayName>
+        <AccountId>773</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B31D159F86750749BAD869CB65D39E6C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b52437f09c885264a74a7224ddae0bf2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94" xmlns:ns3="10d644ba-cf16-43e8-a31a-a6f565d9c224" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a7cbcd1702d69c471f1439a09cbaf55" ns2:_="" ns3:_="">
     <xsd:import namespace="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
@@ -1353,34 +1412,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
+    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
-      <UserInfo>
-        <DisplayName>Helen Browne</DisplayName>
-        <AccountId>773</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D154ECB-7BD7-4B38-A220-236438B72B0E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1397,23 +1448,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
-    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>